<commit_message>
feat(pdf): la pagina de grafica 3D se arma con las tres vistas por separado
Antes entraba una sola imagen con las tres vistas ya compuestas adentro. Los
titulos, si los hubiera, habrian ido dibujados dentro del PNG y con otra
tipografia que el resto del documento.

Ahora la hoja Grafica3D tiene tres recuadros y los titulos son celdas de la
plantilla, con la misma banda naranja que usa la pagina 1 para DATOS CLIENTE o
REPISAS: titulo de pagina, bajada, y uno por imagen. La cotizacion le pide al
configurador cada vista en la medida exacta de su recuadro, asi que ninguna
entra deformada.

Reparte: isometrica y planta arriba, y la vista desde la entrada abajo a todo
el ancho, que es la de campo amplio.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/netlify/functions/cotizacion.xlsx
+++ b/netlify/functions/cotizacion.xlsx
@@ -1652,46 +1652,30 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>334883</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>167974</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>531105</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>384541</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{498F389D-2CE5-4D8E-874B-6B18BA7D0B89}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="2" name="Logo"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8183483" y="800434"/>
-          <a:ext cx="2215522" cy="788067"/>
-        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -1702,25 +1686,19 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>213239</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>138344</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>797027</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>68568</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31768B66-2231-389F-00FC-2119B7D4F418}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="3" name="Isometrica"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1732,10 +1710,74 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8054109" y="1794866"/>
-          <a:ext cx="5785266" cy="4943963"/>
-        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Planta"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Entrada"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -5131,7 +5173,11 @@
       <c r="R7" s="12"/>
     </row>
     <row r="8" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K8" s="108"/>
+      <c r="K8" s="70" t="inlineStr">
+        <is>
+          <t>SIMULACIÓN DEL PROYECTO A REALIZAR</t>
+        </is>
+      </c>
       <c r="L8" s="109"/>
       <c r="M8" s="109"/>
       <c r="N8" s="109"/>
@@ -5159,12 +5205,20 @@
       <c r="Q10" s="5"/>
       <c r="S10" s="12"/>
     </row>
-    <row r="11" spans="11:80" x14ac:dyDescent="0.3">
-      <c r="K11" s="27"/>
+    <row r="11" spans="11:80" x14ac:dyDescent="0.3" ht="21" customHeight="1">
+      <c r="K11" s="70" t="inlineStr">
+        <is>
+          <t>VISTA ISOMÉTRICA</t>
+        </is>
+      </c>
       <c r="L11" s="25"/>
       <c r="M11" s="25"/>
       <c r="N11" s="25"/>
-      <c r="O11" s="25"/>
+      <c r="O11" s="70" t="inlineStr">
+        <is>
+          <t>PLANTA</t>
+        </is>
+      </c>
       <c r="P11" s="25"/>
       <c r="Q11" s="5"/>
       <c r="CB11" s="16"/>
@@ -5188,11 +5242,11 @@
       <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="108"/>
+      <c r="K14" s="25"/>
       <c r="L14" s="109"/>
       <c r="M14" s="109"/>
+      <c r="O14" s="25"/>
       <c r="N14" s="109"/>
-      <c r="O14" s="109"/>
       <c r="P14" s="109"/>
       <c r="Q14" s="110"/>
       <c r="R14" s="12"/>
@@ -5299,8 +5353,12 @@
       <c r="Q25" s="5"/>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K26" s="27"/>
+    <row r="26" spans="11:18" x14ac:dyDescent="0.3" ht="21" customHeight="1">
+      <c r="K26" s="70" t="inlineStr">
+        <is>
+          <t>VISTA DESDE LA ENTRADA</t>
+        </is>
+      </c>
       <c r="L26" s="25"/>
       <c r="M26" s="25"/>
       <c r="N26" s="25"/>
@@ -5466,9 +5524,11 @@
     <mergeCell ref="K24:Q24"/>
     <mergeCell ref="K3:Q3"/>
     <mergeCell ref="K8:Q8"/>
-    <mergeCell ref="K14:Q14"/>
+    <mergeCell ref="K11:N11"/>
+    <mergeCell ref="O11:Q11"/>
     <mergeCell ref="K19:M19"/>
     <mergeCell ref="K21:Q21"/>
+    <mergeCell ref="K26:Q26"/>
     <mergeCell ref="M22:Q22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(plantilla): saca los datos de la cotizacion de muestra de las paginas fijas
Las paginas de marketing quedaron con los datos de la cotizacion que estaba
abierta cuando se armo la plantilla: nombre y telefono de una clienta, las
medidas y los valores de sus repisas, repetidos en las cinco. No se ven porque
la imagen de cada pagina los tapa, pero viajan en el PDF y salen con cualquier
extractor de texto o al copiar y pegar.

Se vacian las filas 9 a 22 en las cinco paginas conservando el formato, mas el
bloque de cliente de la primera, que igual se reescribe en cada cotizacion. Se
mantienen los titulos, el link del portafolio y los de pago.

Comprobado sobre el PDF generado: cero coincidencias del nombre y el telefono en
las siete paginas, y las paginas fijas siguen mostrando su contenido.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/netlify/functions/cotizacion.xlsx
+++ b/netlify/functions/cotizacion.xlsx
@@ -2180,9 +2180,7 @@
       <c r="K9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="102" t="s">
-        <v>45</v>
-      </c>
+      <c r="L9" s="102"/>
       <c r="M9" s="102"/>
       <c r="N9" s="102"/>
       <c r="O9" s="102"/>
@@ -2193,9 +2191,7 @@
       <c r="K10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="87" t="s">
-        <v>7</v>
-      </c>
+      <c r="L10" s="87"/>
       <c r="M10" s="87"/>
       <c r="N10" s="87"/>
       <c r="O10" s="87"/>
@@ -2207,9 +2203,7 @@
       <c r="K11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="L11" s="87" t="s">
-        <v>7</v>
-      </c>
+      <c r="L11" s="87"/>
       <c r="M11" s="87"/>
       <c r="N11" s="87"/>
       <c r="O11" s="87"/>
@@ -2221,9 +2215,7 @@
       <c r="K12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L12" s="87">
-        <v>974139187</v>
-      </c>
+      <c r="L12" s="87"/>
       <c r="M12" s="87"/>
       <c r="N12" s="87"/>
       <c r="O12" s="87"/>
@@ -2234,9 +2226,7 @@
       <c r="K13" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="L13" s="89" t="s">
-        <v>7</v>
-      </c>
+      <c r="L13" s="89"/>
       <c r="M13" s="90"/>
       <c r="N13" s="90"/>
       <c r="O13" s="90"/>
@@ -2831,9 +2821,7 @@
     </row>
     <row r="9" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K9" s="27"/>
-      <c r="L9" s="25" t="s">
-        <v>45</v>
-      </c>
+      <c r="L9" s="25"/>
       <c r="M9" s="25"/>
       <c r="N9" s="25"/>
       <c r="O9" s="25"/>
@@ -2842,9 +2830,7 @@
     </row>
     <row r="10" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K10" s="27"/>
-      <c r="L10" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L10" s="25"/>
       <c r="M10" s="25"/>
       <c r="N10" s="25"/>
       <c r="O10" s="25"/>
@@ -2854,9 +2840,7 @@
     </row>
     <row r="11" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K11" s="27"/>
-      <c r="L11" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L11" s="25"/>
       <c r="M11" s="25"/>
       <c r="N11" s="25"/>
       <c r="O11" s="25"/>
@@ -2866,9 +2850,7 @@
     </row>
     <row r="12" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K12" s="27"/>
-      <c r="L12" s="25">
-        <v>974139187</v>
-      </c>
+      <c r="L12" s="25"/>
       <c r="M12" s="25"/>
       <c r="N12" s="25"/>
       <c r="O12" s="25"/>
@@ -2885,9 +2867,7 @@
       <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="108" t="s">
-        <v>42</v>
-      </c>
+      <c r="K14" s="108"/>
       <c r="L14" s="109"/>
       <c r="M14" s="109"/>
       <c r="N14" s="109"/>
@@ -2906,45 +2886,21 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="11:80" x14ac:dyDescent="0.3">
-      <c r="K16" s="27">
-        <v>1.63</v>
-      </c>
-      <c r="L16" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="25">
-        <v>2</v>
-      </c>
-      <c r="N16" s="25">
-        <v>4</v>
-      </c>
-      <c r="O16" s="25">
-        <v>1</v>
-      </c>
-      <c r="P16" s="25">
-        <v>90000</v>
-      </c>
+      <c r="K16" s="27"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
       <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K17" s="27">
-        <v>1.48</v>
-      </c>
-      <c r="L17" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M17" s="25">
-        <v>1</v>
-      </c>
-      <c r="N17" s="25">
-        <v>2</v>
-      </c>
-      <c r="O17" s="25">
-        <v>1</v>
-      </c>
-      <c r="P17" s="25">
-        <v>50000</v>
-      </c>
+      <c r="K17" s="27"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
       <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="11:18" x14ac:dyDescent="0.3">
@@ -2952,27 +2908,17 @@
       <c r="L18" s="25"/>
       <c r="M18" s="25"/>
       <c r="N18" s="25"/>
-      <c r="O18" s="25">
-        <v>0</v>
-      </c>
-      <c r="P18" s="25">
-        <v>40000</v>
-      </c>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
       <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K19" s="111" t="s">
-        <v>37</v>
-      </c>
+      <c r="K19" s="111"/>
       <c r="L19" s="112"/>
       <c r="M19" s="112"/>
       <c r="N19" s="25"/>
-      <c r="O19" s="25">
-        <v>0</v>
-      </c>
-      <c r="P19" s="25">
-        <v>50000</v>
-      </c>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
       <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="11:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2980,18 +2926,12 @@
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="25">
-        <v>0</v>
-      </c>
-      <c r="P20" s="25">
-        <v>30000</v>
-      </c>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
       <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="11:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K21" s="105" t="s">
-        <v>43</v>
-      </c>
+      <c r="K21" s="105"/>
       <c r="L21" s="106"/>
       <c r="M21" s="106"/>
       <c r="N21" s="106"/>
@@ -3003,9 +2943,7 @@
     <row r="22" spans="11:18" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K22" s="27"/>
       <c r="L22" s="25"/>
-      <c r="M22" s="112">
-        <v>1</v>
-      </c>
+      <c r="M22" s="112"/>
       <c r="N22" s="112"/>
       <c r="O22" s="112"/>
       <c r="P22" s="112"/>
@@ -3303,9 +3241,7 @@
     </row>
     <row r="9" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K9" s="27"/>
-      <c r="L9" s="25" t="s">
-        <v>45</v>
-      </c>
+      <c r="L9" s="25"/>
       <c r="M9" s="25"/>
       <c r="N9" s="25"/>
       <c r="O9" s="25"/>
@@ -3314,9 +3250,7 @@
     </row>
     <row r="10" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K10" s="27"/>
-      <c r="L10" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L10" s="25"/>
       <c r="M10" s="25"/>
       <c r="N10" s="25"/>
       <c r="O10" s="25"/>
@@ -3336,9 +3270,7 @@
     </row>
     <row r="12" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K12" s="27"/>
-      <c r="L12" s="25">
-        <v>974139187</v>
-      </c>
+      <c r="L12" s="25"/>
       <c r="M12" s="25"/>
       <c r="N12" s="25"/>
       <c r="O12" s="25"/>
@@ -3355,9 +3287,7 @@
       <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="108" t="s">
-        <v>42</v>
-      </c>
+      <c r="K14" s="108"/>
       <c r="L14" s="109"/>
       <c r="M14" s="109"/>
       <c r="N14" s="109"/>
@@ -3376,45 +3306,21 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="11:80" x14ac:dyDescent="0.3">
-      <c r="K16" s="27">
-        <v>1.63</v>
-      </c>
-      <c r="L16" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="25">
-        <v>2</v>
-      </c>
-      <c r="N16" s="25">
-        <v>4</v>
-      </c>
-      <c r="O16" s="25">
-        <v>1</v>
-      </c>
-      <c r="P16" s="25">
-        <v>90000</v>
-      </c>
+      <c r="K16" s="27"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
       <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="11:19" x14ac:dyDescent="0.3">
-      <c r="K17" s="27">
-        <v>1.48</v>
-      </c>
-      <c r="L17" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M17" s="25">
-        <v>1</v>
-      </c>
-      <c r="N17" s="25">
-        <v>2</v>
-      </c>
-      <c r="O17" s="25">
-        <v>1</v>
-      </c>
-      <c r="P17" s="25">
-        <v>50000</v>
-      </c>
+      <c r="K17" s="27"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
       <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="11:19" x14ac:dyDescent="0.3">
@@ -3422,27 +3328,17 @@
       <c r="L18" s="25"/>
       <c r="M18" s="25"/>
       <c r="N18" s="25"/>
-      <c r="O18" s="25">
-        <v>0</v>
-      </c>
-      <c r="P18" s="25">
-        <v>40000</v>
-      </c>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
       <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="11:19" x14ac:dyDescent="0.3">
-      <c r="K19" s="111" t="s">
-        <v>37</v>
-      </c>
+      <c r="K19" s="111"/>
       <c r="L19" s="112"/>
       <c r="M19" s="112"/>
       <c r="N19" s="25"/>
-      <c r="O19" s="25">
-        <v>0</v>
-      </c>
-      <c r="P19" s="25">
-        <v>50000</v>
-      </c>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
       <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="11:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -3450,18 +3346,12 @@
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="25">
-        <v>0</v>
-      </c>
-      <c r="P20" s="25">
-        <v>30000</v>
-      </c>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
       <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="11:19" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K21" s="105" t="s">
-        <v>43</v>
-      </c>
+      <c r="K21" s="105"/>
       <c r="L21" s="106"/>
       <c r="M21" s="106"/>
       <c r="N21" s="106"/>
@@ -3473,9 +3363,7 @@
     <row r="22" spans="11:19" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K22" s="27"/>
       <c r="L22" s="25"/>
-      <c r="M22" s="112">
-        <v>1</v>
-      </c>
+      <c r="M22" s="112"/>
       <c r="N22" s="112"/>
       <c r="O22" s="112"/>
       <c r="P22" s="112"/>
@@ -3771,9 +3659,7 @@
     </row>
     <row r="9" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K9" s="27"/>
-      <c r="L9" s="25" t="s">
-        <v>45</v>
-      </c>
+      <c r="L9" s="25"/>
       <c r="M9" s="25"/>
       <c r="N9" s="25"/>
       <c r="O9" s="25"/>
@@ -3782,9 +3668,7 @@
     </row>
     <row r="10" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K10" s="27"/>
-      <c r="L10" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L10" s="25"/>
       <c r="M10" s="25"/>
       <c r="N10" s="25"/>
       <c r="O10" s="25"/>
@@ -3804,9 +3688,7 @@
     </row>
     <row r="12" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K12" s="27"/>
-      <c r="L12" s="25">
-        <v>974139187</v>
-      </c>
+      <c r="L12" s="25"/>
       <c r="M12" s="25"/>
       <c r="N12" s="25"/>
       <c r="O12" s="25"/>
@@ -3823,9 +3705,7 @@
       <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="108" t="s">
-        <v>42</v>
-      </c>
+      <c r="K14" s="108"/>
       <c r="L14" s="109"/>
       <c r="M14" s="109"/>
       <c r="N14" s="109"/>
@@ -3844,45 +3724,21 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="11:80" x14ac:dyDescent="0.3">
-      <c r="K16" s="27">
-        <v>1.63</v>
-      </c>
-      <c r="L16" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="25">
-        <v>2</v>
-      </c>
-      <c r="N16" s="25">
-        <v>4</v>
-      </c>
-      <c r="O16" s="25">
-        <v>1</v>
-      </c>
-      <c r="P16" s="25">
-        <v>90000</v>
-      </c>
+      <c r="K16" s="27"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
       <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K17" s="27">
-        <v>1.48</v>
-      </c>
-      <c r="L17" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M17" s="25">
-        <v>1</v>
-      </c>
-      <c r="N17" s="25">
-        <v>2</v>
-      </c>
-      <c r="O17" s="25">
-        <v>1</v>
-      </c>
-      <c r="P17" s="25">
-        <v>50000</v>
-      </c>
+      <c r="K17" s="27"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
       <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="11:18" x14ac:dyDescent="0.3">
@@ -3890,27 +3746,17 @@
       <c r="L18" s="25"/>
       <c r="M18" s="25"/>
       <c r="N18" s="25"/>
-      <c r="O18" s="25">
-        <v>0</v>
-      </c>
-      <c r="P18" s="25">
-        <v>40000</v>
-      </c>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
       <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K19" s="111" t="s">
-        <v>37</v>
-      </c>
+      <c r="K19" s="111"/>
       <c r="L19" s="112"/>
       <c r="M19" s="112"/>
       <c r="N19" s="25"/>
-      <c r="O19" s="25">
-        <v>0</v>
-      </c>
-      <c r="P19" s="25">
-        <v>50000</v>
-      </c>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
       <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="11:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -3918,18 +3764,12 @@
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="25">
-        <v>0</v>
-      </c>
-      <c r="P20" s="25">
-        <v>30000</v>
-      </c>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
       <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="11:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K21" s="105" t="s">
-        <v>43</v>
-      </c>
+      <c r="K21" s="105"/>
       <c r="L21" s="106"/>
       <c r="M21" s="106"/>
       <c r="N21" s="106"/>
@@ -3941,9 +3781,7 @@
     <row r="22" spans="11:18" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K22" s="27"/>
       <c r="L22" s="25"/>
-      <c r="M22" s="112">
-        <v>1</v>
-      </c>
+      <c r="M22" s="112"/>
       <c r="N22" s="112"/>
       <c r="O22" s="112"/>
       <c r="P22" s="112"/>
@@ -4239,9 +4077,7 @@
     </row>
     <row r="9" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K9" s="27"/>
-      <c r="L9" s="50" t="s">
-        <v>45</v>
-      </c>
+      <c r="L9" s="50"/>
       <c r="M9" s="50"/>
       <c r="N9" s="50"/>
       <c r="O9" s="50"/>
@@ -4250,9 +4086,7 @@
     </row>
     <row r="10" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K10" s="27"/>
-      <c r="L10" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L10" s="25"/>
       <c r="M10" s="25"/>
       <c r="N10" s="25"/>
       <c r="O10" s="25"/>
@@ -4262,9 +4096,7 @@
     </row>
     <row r="11" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K11" s="27"/>
-      <c r="L11" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L11" s="25"/>
       <c r="M11" s="25"/>
       <c r="N11" s="25"/>
       <c r="O11" s="25"/>
@@ -4274,9 +4106,7 @@
     </row>
     <row r="12" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K12" s="27"/>
-      <c r="L12" s="25">
-        <v>974139187</v>
-      </c>
+      <c r="L12" s="25"/>
       <c r="M12" s="25"/>
       <c r="N12" s="25"/>
       <c r="O12" s="25"/>
@@ -4293,9 +4123,7 @@
       <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="108" t="s">
-        <v>42</v>
-      </c>
+      <c r="K14" s="108"/>
       <c r="L14" s="109"/>
       <c r="M14" s="109"/>
       <c r="N14" s="109"/>
@@ -4314,45 +4142,21 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="11:80" x14ac:dyDescent="0.3">
-      <c r="K16" s="27">
-        <v>1.63</v>
-      </c>
-      <c r="L16" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="25">
-        <v>2</v>
-      </c>
-      <c r="N16" s="25">
-        <v>4</v>
-      </c>
-      <c r="O16" s="25">
-        <v>1</v>
-      </c>
-      <c r="P16" s="25">
-        <v>90000</v>
-      </c>
+      <c r="K16" s="27"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
       <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K17" s="27">
-        <v>1.48</v>
-      </c>
-      <c r="L17" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M17" s="25">
-        <v>1</v>
-      </c>
-      <c r="N17" s="25">
-        <v>2</v>
-      </c>
-      <c r="O17" s="25">
-        <v>1</v>
-      </c>
-      <c r="P17" s="25">
-        <v>50000</v>
-      </c>
+      <c r="K17" s="27"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
       <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="11:18" x14ac:dyDescent="0.3">
@@ -4360,27 +4164,17 @@
       <c r="L18" s="25"/>
       <c r="M18" s="25"/>
       <c r="N18" s="25"/>
-      <c r="O18" s="25">
-        <v>0</v>
-      </c>
-      <c r="P18" s="25">
-        <v>40000</v>
-      </c>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
       <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K19" s="111" t="s">
-        <v>37</v>
-      </c>
+      <c r="K19" s="111"/>
       <c r="L19" s="112"/>
       <c r="M19" s="112"/>
       <c r="N19" s="25"/>
-      <c r="O19" s="25">
-        <v>0</v>
-      </c>
-      <c r="P19" s="25">
-        <v>50000</v>
-      </c>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
       <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="11:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4388,18 +4182,12 @@
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="25">
-        <v>0</v>
-      </c>
-      <c r="P20" s="25">
-        <v>30000</v>
-      </c>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
       <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="11:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K21" s="105" t="s">
-        <v>43</v>
-      </c>
+      <c r="K21" s="105"/>
       <c r="L21" s="106"/>
       <c r="M21" s="106"/>
       <c r="N21" s="106"/>
@@ -4411,9 +4199,7 @@
     <row r="22" spans="11:18" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K22" s="27"/>
       <c r="L22" s="25"/>
-      <c r="M22" s="112">
-        <v>1</v>
-      </c>
+      <c r="M22" s="112"/>
       <c r="N22" s="112"/>
       <c r="O22" s="112"/>
       <c r="P22" s="112"/>
@@ -4718,9 +4504,7 @@
     </row>
     <row r="9" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K9" s="27"/>
-      <c r="L9" s="25" t="s">
-        <v>45</v>
-      </c>
+      <c r="L9" s="25"/>
       <c r="M9" s="25"/>
       <c r="N9" s="25"/>
       <c r="O9" s="25"/>
@@ -4729,9 +4513,7 @@
     </row>
     <row r="10" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K10" s="27"/>
-      <c r="L10" s="25" t="s">
-        <v>7</v>
-      </c>
+      <c r="L10" s="25"/>
       <c r="M10" s="25"/>
       <c r="N10" s="25"/>
       <c r="O10" s="25"/>
@@ -4751,9 +4533,7 @@
     </row>
     <row r="12" spans="11:80" x14ac:dyDescent="0.3">
       <c r="K12" s="27"/>
-      <c r="L12" s="25">
-        <v>974139187</v>
-      </c>
+      <c r="L12" s="25"/>
       <c r="M12" s="25"/>
       <c r="N12" s="25"/>
       <c r="O12" s="25"/>
@@ -4770,9 +4550,7 @@
       <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="11:80" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="108" t="s">
-        <v>42</v>
-      </c>
+      <c r="K14" s="108"/>
       <c r="L14" s="109"/>
       <c r="M14" s="109"/>
       <c r="N14" s="109"/>
@@ -4791,45 +4569,21 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="11:80" x14ac:dyDescent="0.3">
-      <c r="K16" s="27">
-        <v>1.63</v>
-      </c>
-      <c r="L16" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M16" s="25">
-        <v>2</v>
-      </c>
-      <c r="N16" s="25">
-        <v>4</v>
-      </c>
-      <c r="O16" s="25">
-        <v>1</v>
-      </c>
-      <c r="P16" s="25">
-        <v>90000</v>
-      </c>
+      <c r="K16" s="27"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
       <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K17" s="27">
-        <v>1.48</v>
-      </c>
-      <c r="L17" s="25">
-        <v>0.48</v>
-      </c>
-      <c r="M17" s="25">
-        <v>1</v>
-      </c>
-      <c r="N17" s="25">
-        <v>2</v>
-      </c>
-      <c r="O17" s="25">
-        <v>1</v>
-      </c>
-      <c r="P17" s="25">
-        <v>50000</v>
-      </c>
+      <c r="K17" s="27"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
       <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="11:18" x14ac:dyDescent="0.3">
@@ -4837,27 +4591,17 @@
       <c r="L18" s="25"/>
       <c r="M18" s="25"/>
       <c r="N18" s="25"/>
-      <c r="O18" s="25">
-        <v>0</v>
-      </c>
-      <c r="P18" s="25">
-        <v>40000</v>
-      </c>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
       <c r="Q18" s="5"/>
     </row>
     <row r="19" spans="11:18" x14ac:dyDescent="0.3">
-      <c r="K19" s="111" t="s">
-        <v>37</v>
-      </c>
+      <c r="K19" s="111"/>
       <c r="L19" s="112"/>
       <c r="M19" s="112"/>
       <c r="N19" s="25"/>
-      <c r="O19" s="25">
-        <v>0</v>
-      </c>
-      <c r="P19" s="25">
-        <v>50000</v>
-      </c>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
       <c r="Q19" s="5"/>
     </row>
     <row r="20" spans="11:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4865,18 +4609,12 @@
       <c r="L20" s="25"/>
       <c r="M20" s="25"/>
       <c r="N20" s="25"/>
-      <c r="O20" s="25">
-        <v>0</v>
-      </c>
-      <c r="P20" s="25">
-        <v>30000</v>
-      </c>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
       <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="11:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="K21" s="105" t="s">
-        <v>43</v>
-      </c>
+      <c r="K21" s="105"/>
       <c r="L21" s="106"/>
       <c r="M21" s="106"/>
       <c r="N21" s="106"/>
@@ -4888,9 +4626,7 @@
     <row r="22" spans="11:18" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="K22" s="27"/>
       <c r="L22" s="25"/>
-      <c r="M22" s="112">
-        <v>1</v>
-      </c>
+      <c r="M22" s="112"/>
       <c r="N22" s="112"/>
       <c r="O22" s="112"/>
       <c r="P22" s="112"/>

</xml_diff>